<commit_message>
Added and fixed bolckchain
</commit_message>
<xml_diff>
--- a/Matrusri_Engineering_college_Certificates.xlsx
+++ b/Matrusri_Engineering_college_Certificates.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -100,6 +100,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -576,84 +579,646 @@
           <t>GAUTAM BABEL JAIN</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="3" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O7" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:09:55.622314</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORKS: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: S (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS: S ()</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_090315_Mist.jpg</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:33:29.427589</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>160822733176</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>OSMANIA UNIVERSITY</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>B.E.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>C.S.E.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>B.E. Semester 5</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>8.67</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>29/05/2025</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>1040471</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>OSMANIA UNIVERSITY</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>SOFTWARE ENGINEERIN: A (); PRINCIPLES OF PROGRAM.LAN: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORK: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: S (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Matrusri_Engineering_college_20251213_003528_WhatsApp_Image_2025-12-12_at_9.12.29_PM.jpeg</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORKS: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: S (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS: S ()</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_090315_Mist.jpg</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>2025-12-13</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-12T19:05:36.570012</t>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T03:33:29.427589</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
removed verificatin page dropdown
</commit_message>
<xml_diff>
--- a/Matrusri_Engineering_college_Certificates.xlsx
+++ b/Matrusri_Engineering_college_Certificates.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -100,9 +100,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -579,8 +576,10 @@
           <t>GAUTAM BABEL JAIN</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
-        <v>160822733176</v>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>160822733176</t>
+        </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -597,25 +596,35 @@
           <t>C.S.E.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>5</v>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>B.E. Semester 5</t>
         </is>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>8.67</v>
-      </c>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>8.67</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>29/05/2025</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n">
-        <v>1040471</v>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>1040471</t>
+        </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
@@ -624,12 +633,12 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: B (); COMPUTER NETWORKS LAB: S ()</t>
+          <t>SOFTWARE ENGINEERIN: A (); PRINCIPLES OF PROGRAM.LAN: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORK: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Matrusri_Engineering_college_20251213_083943_Screenshot_2025-12-12_154733.png</t>
+          <t>Matrusri_Engineering_college_20251213_114322_WhatsApp_Image_2025-12-12_at_9.12.29_PM.jpeg</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
@@ -639,94 +648,12 @@
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>2025-12-13T03:09:55.622314</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Shourya Hagaldivte</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>160822733099</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>OSMANIA UNIVERSITY</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>B.E.</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>C.S.E.</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>B.E. Semester 5</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>8.21</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>29/05/2025</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>1040471</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>OSMANIA UNIVERSITY</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>SOFTWARE ENGINEERING: A (); PRINCIPLES OF PROGRAM.LANG.: A (); AUTOMATA LANGU.AND COMPUTATION: A (); ARTIFICIAL INTELLIGENCE: B (); COMPUTER NETWORKS: A (); DATA SCIENCE: B (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>Matrusri_Engineering_college_20251213_092117_Screenshot_2025-12-12_154733.png</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>2025-12-13</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>2025-12-13T03:51:30.372652</t>
+          <t>2025-12-13T06:13:35.710489</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P3"/>
+  <autoFilter ref="A1:P2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Loosened the sha256 hash algo
</commit_message>
<xml_diff>
--- a/Matrusri_Engineering_college_Certificates.xlsx
+++ b/Matrusri_Engineering_college_Certificates.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$P$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -100,6 +100,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -576,84 +579,228 @@
           <t>GAUTAM BABEL JAIN</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="3" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERIN: A (); PRINCIPLES OF PROGRAM.LAN: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORK: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_114322_WhatsApp_Image_2025-12-12_at_9.12.29_PM.jpeg</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T06:13:35.710489</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>160822733176</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>B.E.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>C.S.E.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>B.E. Semester 5</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>29/05/2025</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>1040471</v>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>OSMANIA UNIVERSITY</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERIN: A (); PRINCIPLES OF PROGRAM.LAN: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORK: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: S (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_133556_Original.jpg</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>2025-12-13T08:06:10.513199</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>GAUTAM BABEL JAIN</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>160822733176</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>OSMANIA UNIVERSITY</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>B.E.</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>C.S.E.</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>B.E. Semester 5</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>8.67</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>29/05/2025</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>1040471</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>OSMANIA UNIVERSITY</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>SOFTWARE ENGINEERIN: A (); PRINCIPLES OF PROGRAM.LAN: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORK: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: A (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Matrusri_Engineering_college_20251213_114322_WhatsApp_Image_2025-12-12_at_9.12.29_PM.jpeg</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>SOFTWARE ENGINEERIN: A (); PRINCIPLES OF PROGRAM.LAN: A (); AUTOMATA LANGU.AND COMPUTATION: B (); ARTIFICIAL INTELLIGENCE: A (); COMPUTER NETWORK: B (); DATA SCIENCE: A (); SOFTWARE ENGINEERING LAB: S (); ARTIFICIAL INTELLIGENCE LAB: S (); COMPUTER NETWORKS LAB: S ()</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Matrusri_Engineering_college_20251213_134339_Original.jpg</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>2025-12-13</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>2025-12-13T06:13:35.710489</t>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T08:13:58.614686</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>